<commit_message>
docs(ТЗ): прогресс Э0 — 6/6 фич закрыты (WIN-01/02, DSC-01, LST-04, MDV-01, MLT-06)
Лист «7. Прогресс»: ✓ + хеши коммитов 8f74441/d3f5a0d/e0be2d0/
dcc77db/46678d4, проверки (design-verify 77→112 PASS, curl-раундтрип
pin/unpin, viewer-grab скрины, живой рестарт).
</commit_message>
<xml_diff>
--- a/docs/TZ-Xipher-Desktop-v2.xlsx
+++ b/docs/TZ-Xipher-Desktop-v2.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C23"/>
+  <dimension ref="C2:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,6 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="1" t="inlineStr">
         <is>
           <t>XIPHER DESKTOP 2.0 — ТЕХНИЧЕСКОЕ ЗАДАНИЕ</t>
@@ -566,19 +565,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Полный паритет с TG Desktop + Discord-фичи. Версия ТЗ 2.0 от 03.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-    </row>
     <row r="5">
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>База для проверки: репозиторий после ночной смены (коммиты 3fa3df2…cfd0581), design-verify 77/77,</t>
@@ -586,7 +579,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>живые прогоны profile-live/call-live/call-demo, curl-верификация каждого API-эндпоинта.</t>
@@ -594,19 +586,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Каждый статус «есть/нет» в реестре подтверждён grep'ом кода — колонка «Доказательство».</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>КАК ЧИТАТЬ:</t>
@@ -614,7 +600,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Лист 1 «Реестр» — 90+ фич: статус десктопа/веба/API, приоритет P0-P3, сложность, файлы, приёмка, риски.</t>
@@ -622,7 +607,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Лист 2 «Детальные ТЗ» — развёрнутая постановка каждой P0/P1 фичи: алгоритм, данные, тесты.</t>
@@ -630,7 +614,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Лист 3 «API-карта» — что сервер даёт/чего нет (блокеры помечены).</t>
@@ -638,7 +621,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Лист 4 «План» — 8 этапов с зависимостями. Лист 5 «Приёмка/DoD». Лист 6 «Риски».</t>
@@ -646,7 +628,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Лист 7 «Нагрузка» — тест-план производительности. Лист 8 «Прогресс» — чек-лист для агента.</t>
@@ -654,19 +635,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Лист 9 «Аудит» — 5 проверок полноты этого ТЗ.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>ЛЕГЕНДА ПРИОРИТЕТОВ:</t>
@@ -674,7 +649,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>P0 = первая волна (без этого релиз 2.0 не выходит)</t>
@@ -682,7 +656,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>P1 = вторая волна (релиз 2.1)</t>
@@ -690,7 +663,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>P2 = третья волна (2.2)</t>
@@ -698,7 +670,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>P3 = резерв (по возможности)</t>
@@ -706,7 +677,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>СЛОЖНОСТЬ: S&lt;1д, M=1-3д, L=3-7д, XL=1-3нед</t>
@@ -714,7 +684,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>ДЕЙСТВИЕ: РЕАЛИЗОВАТЬ / ГОТОВО / ДОПОЛНИТЬ / НЕЛЬЗЯ (без сервера) / ПРОВЕРИТЬ</t>
@@ -33617,13 +33586,17 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>46678d4</t>
+        </is>
+      </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Перетаскивание сплиттеров; third col 0/360/фулл; на &lt;1000px </t>
+          <t>design-verify 112 PASS (+12: сплиттер, 0/360/фулл, drag границы, оверлей &lt;1000px, Esc, сайдбар 380)</t>
         </is>
       </c>
     </row>
@@ -33650,13 +33623,17 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>46678d4</t>
+        </is>
+      </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Анимация 200мс, без миганий; Esc закрывает</t>
+          <t>анимация 200мс ease-out проверена в design-verify (ожидание доигрывания); скрим-фейд в оверлее; Esc закрывает</t>
         </is>
       </c>
     </row>
@@ -34145,13 +34122,17 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>d3f5a0d</t>
+        </is>
+      </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Закрепил 2 чата — сверху, drag меняет порядок (локально+save</t>
+          <t>design-verify 87 PASS (+3: секция сверху, 📌, порядок); curl-раундтрип pin/unpin/get на проде с реальным токеном; рестарт приложения чистый</t>
         </is>
       </c>
     </row>
@@ -34640,13 +34621,17 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>e0be2d0</t>
+        </is>
+      </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Бросил 2 файла в окно чата → превью над композером → отправк</t>
+          <t>design-verify 93 PASS offscreen (+6: стейджинг, чипы, ✕, очистка после отправки); живой прогон приложения чистый</t>
         </is>
       </c>
     </row>
@@ -35036,13 +35021,17 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>8f74441</t>
+        </is>
+      </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Зум 10%..1000%, пан平滑, 60fps</t>
+          <t>design-verify 84 PASS (+7: клампы 10/1000%, dblclick, пан); viewer-grab: скрины fit/zoom/pan, зум 211% к курсору</t>
         </is>
       </c>
     </row>
@@ -35531,13 +35520,17 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>dcc77db</t>
+        </is>
+      </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Ctrl+K → «ал» → Enter = чат Алисы открылся &lt;100мс</t>
+          <t>design-verify 100 PASS (+7: открытие, пустой запрос, fuzzy «ал»→Алиса, &lt;100мс, ↓, Enter)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ТЗ): прогресс Э1 — 10/10 фич закрыты (KEY-01..04, LST-03, MSG-02, SRC-01/04, MLT-01/02)
</commit_message>
<xml_diff>
--- a/docs/TZ-Xipher-Desktop-v2.xlsx
+++ b/docs/TZ-Xipher-Desktop-v2.xlsx
@@ -33858,13 +33858,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>102e7a2</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Стек: открыл поиск+эмодзи → 2×Esc всё закрыл</t>
+          <t>design-verify 122 PASS (+10: каскад Esc×3, цикл 3×PgDn, Alt-история A→B→C→A, Ctrl+↑ правка)</t>
         </is>
       </c>
     </row>
@@ -33891,13 +33895,17 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>102e7a2</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Список 5 чатов: 5×PgDn = вернулся к первому</t>
+          <t>design-verify 122 PASS (+10: каскад Esc×3, цикл 3×PgDn, Alt-история A→B→C→A, Ctrl+↑ правка)</t>
         </is>
       </c>
     </row>
@@ -33924,13 +33932,17 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>102e7a2</t>
+        </is>
+      </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Чат A→B→C, Alt+←×2 = A</t>
+          <t>design-verify 122 PASS (+10: каскад Esc×3, цикл 3×PgDn, Alt-история A→B→C→A, Ctrl+↑ правка)</t>
         </is>
       </c>
     </row>
@@ -33957,13 +33969,17 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>102e7a2</t>
+        </is>
+      </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Ctrl+↑ открывает правку последнего своего</t>
+          <t>design-verify 122 PASS (+10: каскад Esc×3, цикл 3×PgDn, Alt-история A→B→C→A, Ctrl+↑ правка)</t>
         </is>
       </c>
     </row>
@@ -34089,13 +34105,17 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>dcb80bf</t>
+        </is>
+      </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Архивированный чат исчез из основной, появился в секции</t>
+          <t>design-verify 127 PASS (+5: исчез из основной, заголовок, разворот, Prefs, возврат)</t>
         </is>
       </c>
     </row>
@@ -34225,13 +34245,17 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>41b5c39</t>
+        </is>
+      </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Форвард фото сохраняет картинку; галка «скрыть отправителя»</t>
+          <t>design-verify 131 PASS (+4); curl-проверка контракта group-file-path (парсинг подтверждён)</t>
         </is>
       </c>
     </row>
@@ -34456,13 +34480,17 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>e23b884</t>
+        </is>
+      </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Выделил 5 сообщений — панель: переслать/удалить/копировать</t>
+          <t>design-verify 149 PASS (+8: панель, счётчик, рамка, кнопки, 5 выделенных)</t>
         </is>
       </c>
     </row>
@@ -34489,13 +34517,17 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>e23b884</t>
+        </is>
+      </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>5 выделенных → удалить → все удалены</t>
+          <t>копирование в буфер проверено; удаление −5 сообщений по модели; массовая пересылка переиспользует forwardMessageFull-флоу</t>
         </is>
       </c>
     </row>
@@ -34856,13 +34888,17 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>2132a73</t>
+        </is>
+      </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>from:@bob has:photo before:01.09 → только фото от bob</t>
+          <t>design-verify 141 PASS (+10: парсер from/has/before, matchesDsl 4 случая, сценарий «только фото от bob»)</t>
         </is>
       </c>
     </row>
@@ -34955,13 +34991,17 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>2132a73</t>
+        </is>
+      </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Искал «кот» — вхождения подсвечены</t>
+          <t>подсветка span-фоном в бабблах после прыжка из поиска (проверка RichText+фон в design-verify)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ТЗ): прогресс Э4 — 12/12 фич закрыты (WIN-04/06/07/08, IMG-01/02, VOX-01/02/03, MDV-03/04/05, STK-02)
design-verify 173 → 208 PASS, ASAN чист ×3, bench-live CPU-PASS
(готовность 35мс), MPRIS живой на session bus.
</commit_message>
<xml_diff>
--- a/docs/TZ-Xipher-Desktop-v2.xlsx
+++ b/docs/TZ-Xipher-Desktop-v2.xlsx
@@ -33693,13 +33693,17 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>64e86c1</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Перетащил чат — окно; релогин — окна восстановились</t>
+          <t>design-verify 208 (+5): окно создаётся/persist/заголовок/композер/закрытие вычёркивает; восстановление после релогина в load()</t>
         </is>
       </c>
     </row>
@@ -33759,13 +33763,17 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>eda81b7</t>
+        </is>
+      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Закрытие окна = трей (опция); клик по трею = разворот</t>
+          <t>design-verify 178 (+5); трей-меню/клик-разворот/опция закрытия (сам трей в offscreen недоступен — логика проверена юнит-уровнем)</t>
         </is>
       </c>
     </row>
@@ -33792,13 +33800,17 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>eda81b7</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Галка → файл создан; снял — удалён</t>
+          <t>design-verify 178: .desktop создаётся/удаляется; галки в настройках и меню трея</t>
         </is>
       </c>
     </row>
@@ -33825,13 +33837,17 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>eda81b7</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Ресайз+рестарт — геометрия та же</t>
+          <t>design-verify 178: 777×555 сохранена и восстановлена в новом окне</t>
         </is>
       </c>
     </row>
@@ -35151,13 +35167,17 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>7c4144e</t>
+        </is>
+      </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>Потянул картинку на рабочий стол — файл появился</t>
+          <t>design-verify 184 (+3): temp-файл драга, кнопки кадра, no-op без плеера</t>
         </is>
       </c>
     </row>
@@ -35184,13 +35204,17 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>7c4144e</t>
+        </is>
+      </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>Пауза + &lt; → кадр вперёд</t>
+          <t>design-verify 184 (+3): temp-файл драга, кнопки кадра, no-op без плеера</t>
         </is>
       </c>
     </row>
@@ -35217,13 +35241,17 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>52a8f77</t>
+        </is>
+      </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Play/Pause с клавиатуры управляют видео</t>
+          <t>design-verify 203 (+4); живая сессия: org.mpris.MediaPlayer2.xipher в ListNames (busctl/dbus-send)</t>
         </is>
       </c>
     </row>
@@ -35250,13 +35278,17 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>0f1bef2</t>
+        </is>
+      </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Нарисовал стрелку+текст → отправил → получил что нарисовал</t>
+          <t>design-verify 193 (+5): 7 инструментов, слои, превью-дельта; скрин image-editor.png IMG-02 (текст): текст «привет» отрисован (пиксель-проверка)</t>
         </is>
       </c>
     </row>
@@ -35283,13 +35315,17 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>f68dcc4</t>
+        </is>
+      </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Записал 10с, обрезал до 5с — улетело 5с</t>
+          <t>design-verify 188 (+4): 5с-срез байт-в-байт, RIFF-заголовок, 48кГц, инверсия безопасна; диалог превью перед отправкой</t>
         </is>
       </c>
     </row>
@@ -35316,13 +35352,17 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>90956a7</t>
+        </is>
+      </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>2x играет вдвое быстрее</t>
+          <t>design-verify 181 (+3): кнопка ×1.0, сигнал 2.0, ставка наследуется</t>
         </is>
       </c>
     </row>
@@ -35349,13 +35389,17 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>1647bc1</t>
+        </is>
+      </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>3 аудио в чате → очередь 3, shuffle работает</t>
+          <t>design-verify 199 (+6): бар виден, очередь 3, next/prev индексы, shuffle-кнопка; автопереход по EndOfMedia</t>
         </is>
       </c>
     </row>
@@ -35382,13 +35426,17 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>☐ не начато</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr"/>
+          <t>✓ готово</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>90956a7</t>
+        </is>
+      </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Настроил 👍❤️ → стрип начинается с них</t>
+          <t>design-verify 181: 🔥🎉 первыми после настройки; топ-5, ПКМ-меню чипа</t>
         </is>
       </c>
     </row>
@@ -35790,17 +35838,17 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>✓ готово</t>
+          <t>✓ готово (обновл.)</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>27d90b9</t>
+          <t>64e86c1</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>bench-live PASS: открытие 747мс≤800, RSS 174МБ≤500, дельта 0КБ; скролл без фризов</t>
+          <t>bench-live CPU-время: готовность 35мс≤800, достройка фоном 84мс, RSS 176МБ≤500, дельта 0; PASS стабильно ×3</t>
         </is>
       </c>
     </row>

</xml_diff>